<commit_message>
Ny version av läget i Dalarna
</commit_message>
<xml_diff>
--- a/Data/arbetsloshet_kommun.xlsx
+++ b/Data/arbetsloshet_kommun.xlsx
@@ -56,7 +56,7 @@
     <t xml:space="preserve">arbetslöshet</t>
   </si>
   <si>
-    <t xml:space="preserve">2026M06</t>
+    <t xml:space="preserve">2026M07</t>
   </si>
   <si>
     <t xml:space="preserve">2-4</t>
@@ -527,7 +527,7 @@
         <v>14</v>
       </c>
       <c r="H2" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
@@ -614,7 +614,7 @@
         <v>14</v>
       </c>
       <c r="H5" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="I5" t="s">
         <v>15</v>
@@ -643,7 +643,7 @@
         <v>14</v>
       </c>
       <c r="H6" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="I6" t="s">
         <v>15</v>
@@ -672,7 +672,7 @@
         <v>14</v>
       </c>
       <c r="H7" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
@@ -701,7 +701,7 @@
         <v>14</v>
       </c>
       <c r="H8" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I8" t="s">
         <v>15</v>
@@ -730,7 +730,7 @@
         <v>14</v>
       </c>
       <c r="H9" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="I9" t="s">
         <v>15</v>
@@ -759,7 +759,7 @@
         <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="I10" t="s">
         <v>15</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="H11" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -817,7 +817,7 @@
         <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="I12" t="s">
         <v>36</v>
@@ -846,7 +846,7 @@
         <v>14</v>
       </c>
       <c r="H13" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -904,7 +904,7 @@
         <v>14</v>
       </c>
       <c r="H15" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="I15" t="s">
         <v>36</v>
@@ -933,7 +933,7 @@
         <v>14</v>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="I16" t="s">
         <v>36</v>

</xml_diff>